<commit_message>
Bugfixes, template updates (#98)
Backend:
Discriminate on the metadata label when duplicate typed nodes
Register value nodes so other properties can be added to them

Flowcell:
Fix typos, trailing whitespace
Change bad predicate "Substrate" with "hasSubstrate"
Fix VolumeFlowRate comments creating a separate node
Make substrate thickness comments clearer

Electrolysis:
Fix bad pH unit
Fix typos, trailing whitespace
</commit_message>
<xml_diff>
--- a/test/data/electrolysis_excel_schema.xlsx
+++ b/test/data/electrolysis_excel_schema.xlsx
@@ -859,7 +859,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>0.1.2</t>
+          <t>0.1.3</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1290,7 +1290,7 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Negative electrode coating active material particle size (leave blanc for films)</t>
+          <t>Negative electrode coating active material particle size (leave blank for films)</t>
         </is>
       </c>
       <c r="B29" s="8" t="n">
@@ -1926,7 +1926,7 @@
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>Positive electrode coating active material mean particle size (leave blanc for films)</t>
+          <t>Positive electrode coating active material mean particle size (leave blank for films)</t>
         </is>
       </c>
       <c r="B54" s="12" t="n">
@@ -2498,7 +2498,7 @@
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Catholyte solute A molarity </t>
+          <t>Catholyte solute A molarity</t>
         </is>
       </c>
       <c r="B77" s="16" t="n">
@@ -2572,7 +2572,7 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Catholyte volume  </t>
+          <t>Catholyte volume</t>
         </is>
       </c>
       <c r="B80" s="4" t="n">
@@ -3340,7 +3340,7 @@
     <row r="112">
       <c r="A112" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anolyte solute A molarity </t>
+          <t>Anolyte solute A molarity</t>
         </is>
       </c>
       <c r="B112" s="16" t="n">
@@ -3414,7 +3414,7 @@
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anolyte volume  </t>
+          <t>Anolyte volume</t>
         </is>
       </c>
       <c r="B115" s="4" t="n">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="C120" s="16" t="inlineStr">
         <is>
-          <t>No Unit</t>
+          <t>unitless</t>
         </is>
       </c>
       <c r="D120" s="16" t="inlineStr">
@@ -3914,7 +3914,7 @@
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>Membrane type  (BilayerMembrane or leave blanc)</t>
+          <t>Membrane type  (BilayerMembrane or leave blank)</t>
         </is>
       </c>
       <c r="B136" s="5" t="inlineStr">
@@ -4356,7 +4356,7 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>Cell case type (FlowCell or leave blanc)</t>
+          <t>Cell case type (FlowCell or leave blank)</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
@@ -4384,7 +4384,7 @@
     <row r="155">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>Negative electrode gas compartment (FlowField or leave blanc)</t>
+          <t>Negative electrode gas compartment (FlowField or leave blank)</t>
         </is>
       </c>
       <c r="B155" s="5" t="inlineStr">
@@ -4570,7 +4570,7 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>Anolyte compartement volume</t>
+          <t>Anolyte compartment volume</t>
         </is>
       </c>
       <c r="B162" s="4" t="n">
@@ -4702,7 +4702,7 @@
     <row r="167">
       <c r="A167" s="5" t="inlineStr">
         <is>
-          <t>Positive electrode gas compartment (FlowField or leave blanc)</t>
+          <t>Positive electrode gas compartment (FlowField or leave blank)</t>
         </is>
       </c>
       <c r="B167" s="5" t="inlineStr">
@@ -5256,7 +5256,7 @@
     <row r="2">
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">If the item is listed here without unique ID (e.g. R2032), this means the item is already ontologized in BattInFo ontology. No additional ID is required. </t>
+          <t>If the item is listed here without unique ID (e.g. R2032), this means the item is already ontologized in BattInFo ontology. No additional ID is required.</t>
         </is>
       </c>
     </row>
@@ -5846,7 +5846,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Fumasep FAA by Fumtech (AEM)</t>
+          <t>Fumasep FAA by Fumatech (AEM)</t>
         </is>
       </c>
     </row>
@@ -5889,7 +5889,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teflon by Chemours (PTFE), Polyflon by Daikin (PTFE), </t>
+          <t>Teflon by Chemours (PTFE), Polyflon by Daikin (PTFE),</t>
         </is>
       </c>
     </row>
@@ -6091,7 +6091,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas </t>
+          <t>Gas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix solute solvent nesting, update expected
</commit_message>
<xml_diff>
--- a/test/data/electrolysis_excel_schema.xlsx
+++ b/test/data/electrolysis_excel_schema.xlsx
@@ -1182,7 +1182,7 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Negative electrode optional microstructral/physical parameters</t>
+          <t>Negative electrode optional microstructural/physical parameters</t>
         </is>
       </c>
       <c r="B27" s="7" t="n"/>
@@ -1756,7 +1756,7 @@
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>Positive electrode coating  thickness</t>
+          <t>Positive electrode coating thickness</t>
         </is>
       </c>
       <c r="B52" s="12" t="n">
@@ -2099,7 +2099,7 @@
       <c r="E67" s="4" t="n"/>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-Gas</t>
+          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-type|Gas</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2149,7 @@
       <c r="E69" s="4" t="n"/>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-Gas</t>
+          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-type|Gas</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       <c r="E93" s="4" t="n"/>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolventA-schema:manufacturer</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       <c r="E94" s="16" t="n"/>
       <c r="F94" s="16" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolventA-schema:productID</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentA-schema:productID</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       <c r="E95" s="4" t="n"/>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolventB-schema:manufacturer</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       <c r="E96" s="16" t="n"/>
       <c r="F96" s="16" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSolventB-schema:productID</t>
+          <t>hasCatholyte-hasSolvent-hasConstituentB-schema:productID</t>
         </is>
       </c>
     </row>
@@ -2785,14 +2785,14 @@
       <c r="E97" s="4" t="n"/>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSoluteA-schema:manufacturer</t>
+          <t>hasCatholyte-hasSolute-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
         <is>
-          <t>Catholyte solute A manufacturer productD</t>
+          <t>Catholyte solute A manufacturer product ID</t>
         </is>
       </c>
       <c r="B98" s="16" t="n">
@@ -2807,7 +2807,7 @@
       <c r="E98" s="16" t="n"/>
       <c r="F98" s="16" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSoluteA-schema:productID</t>
+          <t>hasCatholyte-hasSolute-hasConstituentA-schema:productID</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2827,7 @@
       <c r="E99" s="4" t="n"/>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSoluteB-schema:manufacturer</t>
+          <t>hasCatholyte-hasSolute-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
     </row>
@@ -2847,7 +2847,7 @@
       <c r="E100" s="16" t="n"/>
       <c r="F100" s="16" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasSoluteB-schema:productID</t>
+          <t>hasCatholyte-hasSolute-hasConstituentB-schema:productID</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
       <c r="E102" s="4" t="n"/>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-Gas</t>
+          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-type|Gas</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       <c r="E104" s="4" t="n"/>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-Gas</t>
+          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-type|Gas</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       <c r="E128" s="4" t="n"/>
       <c r="F128" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-schema:manufacturer</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       <c r="E129" s="16" t="n"/>
       <c r="F129" s="16" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-schema:productID</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentA-schema:productID</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       <c r="E130" s="4" t="n"/>
       <c r="F130" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-schema:manufacturer</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
     </row>
@@ -3539,7 +3539,7 @@
       <c r="E131" s="16" t="n"/>
       <c r="F131" s="16" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolvent-schema:productID</t>
+          <t>hasAnolyte-hasSolvent-hasConstituentB-schema:productID</t>
         </is>
       </c>
     </row>
@@ -3563,14 +3563,14 @@
       <c r="E132" s="4" t="n"/>
       <c r="F132" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-schema:manufacturer</t>
+          <t>hasAnolyte-hasSolute-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="16" t="inlineStr">
         <is>
-          <t>Anolyte solute A manufacturer productD</t>
+          <t>Anolyte solute A manufacturer product ID</t>
         </is>
       </c>
       <c r="B133" s="16" t="n">
@@ -3585,7 +3585,7 @@
       <c r="E133" s="16" t="n"/>
       <c r="F133" s="16" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-schema:productID</t>
+          <t>hasAnolyte-hasSolute-hasConstituentA-schema:productID</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       <c r="E134" s="4" t="n"/>
       <c r="F134" s="4" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-schema:manufacturer</t>
+          <t>hasAnolyte-hasSolute-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
     </row>
@@ -3625,7 +3625,7 @@
       <c r="E135" s="16" t="n"/>
       <c r="F135" s="16" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasSolute-schema:productID</t>
+          <t>hasAnolyte-hasSolute-hasConstituentB-schema:productID</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>Membrane type</t>
+          <t>Membrane type (BilayerMembrane or leave blank)</t>
         </is>
       </c>
       <c r="B138" s="5" t="inlineStr">
@@ -3682,11 +3682,7 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E138" s="5" t="inlineStr">
-        <is>
-          <t>BilayerMembrane or leave blank</t>
-        </is>
-      </c>
+      <c r="E138" s="5" t="n"/>
       <c r="F138" s="5" t="inlineStr">
         <is>
           <t>hasSeparator</t>
@@ -3908,7 +3904,7 @@
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>Membrane A area specific conductivity</t>
+          <t>Membrane A conductivity</t>
         </is>
       </c>
       <c r="B148" s="4" t="n">
@@ -3934,7 +3930,7 @@
     <row r="149">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>Membrane B area specific conductivity</t>
+          <t>Membrane B conductivity</t>
         </is>
       </c>
       <c r="B149" s="5" t="n">

</xml_diff>